<commit_message>
added search filter and edit button
</commit_message>
<xml_diff>
--- a/static/excel/allInvoices.xlsx
+++ b/static/excel/allInvoices.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,35 +455,25 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>invoice_email</t>
+          <t>invoice_comments</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>invoice_comments</t>
+          <t>product_name</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>product_name</t>
+          <t>product_price</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>product_price</t>
+          <t>product_quantity</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>product_unit</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>product_amount</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>invoice_total</t>
         </is>
@@ -491,45 +481,150 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45696</v>
+        <v>45697</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ss</t>
+          <t>saquib</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>99999999</t>
+          <t>9137768472</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>mohdsaquib91377@gmail.com</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Upma mix</t>
-        </is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>product2</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>500</v>
       </c>
       <c r="H2" t="n">
-        <v>90</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>100 g</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" t="n">
-        <v>90</v>
+        <v>3</v>
+      </c>
+      <c r="I2" t="n">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>45697</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>saquib</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>9137768472</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>producst3</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>3500</v>
+      </c>
+      <c r="H3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I3" t="n">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>45697</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>bilal khan</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>9137768472</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>salam namaste</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>45697</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>obaid khan</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>989898985</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>nike</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>76898987769</v>
+      </c>
+      <c r="H5" t="n">
+        <v>887</v>
+      </c>
+      <c r="I5" t="n">
+        <v>68209402151103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>